<commit_message>
wszystko dziala ale spruta jak zwykle
</commit_message>
<xml_diff>
--- a/myapp/app/templates/excel-blocking.xlsx
+++ b/myapp/app/templates/excel-blocking.xlsx
@@ -129,7 +129,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.7"/>
@@ -148,20 +148,13 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0"/>
-      <c r="C2" s="0"/>
+      <c r="B2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0"/>
-      <c r="C3" s="0"/>
+      <c r="B3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0"/>
-      <c r="C4" s="0"/>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0"/>
-      <c r="C5" s="0"/>
+      <c r="B4" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>